<commit_message>
feat: enrich banking product catalogue
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/banking_products.xlsx
+++ b/data/banking_products.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,31 @@
           <t>target_customer</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>minimum_income</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>age_requirement</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>salary_domiciliation_required</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>included_services</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>key_conditions</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -495,6 +520,29 @@
           <t>particulares</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>18+</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Cartão de débito; acesso à aplicação; transferências nacionais</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Comissão mensal de manutenção; abertura mediante identificação válida</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +574,29 @@
           <t>particulares</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>18+</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Gestor dedicado; cartão premium; transferências internacionais</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Requer domiciliação de salário e rendimento mensal mínimo de 1500 euros</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -557,6 +628,29 @@
           <t>particulares</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>750</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>18+</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cashback de 1,5%; pagamentos contactless; cartão virtual</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Cashback sujeito a categorias e limites definidos no preçário</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -588,6 +682,29 @@
           <t>estudantes</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Cartão de débito; acesso à aplicação; notificações de movimentos</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>É necessário comprovar a condição de estudante</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -617,6 +734,29 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>viajantes</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>18+</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Cashback de 0,5%; seguro de viagem; pagamentos em moeda estrangeira</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Seguro sujeito às condições da apólice; requer análise de elegibilidade</t>
         </is>
       </c>
     </row>

</xml_diff>